<commit_message>
forgot to upload all my DWSIM projects
I reference these in quite a few notes, so I want to have them on hand
</commit_message>
<xml_diff>
--- a/Excel Projects/Candle Making More Realistic.xlsx
+++ b/Excel Projects/Candle Making More Realistic.xlsx
@@ -1,22 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\wille\Desktop\Excel Projects\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\wille\Desktop\Projects-And-Code-Will-Martin\Excel Projects\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5CA267BA-3967-4692-97DC-36FE3AB69E4A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3BECD460-7D7B-4B25-949B-B57CF01DEF99}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-96" yWindow="-96" windowWidth="23232" windowHeight="12552" xr2:uid="{EB9295E0-2A09-4C6A-B14D-2AA5A95FE70B}"/>
+    <workbookView xWindow="11520" yWindow="0" windowWidth="11520" windowHeight="12360" xr2:uid="{EB9295E0-2A09-4C6A-B14D-2AA5A95FE70B}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="191029"/>
-  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -300,10 +299,10 @@
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1"/>
     <xf numFmtId="44" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -658,7 +657,7 @@
   <sheetData>
     <row r="1" spans="1:5" ht="14.4" customHeight="1" x14ac:dyDescent="0.55000000000000004"/>
     <row r="3" spans="1:5" ht="14.4" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A3" s="18" t="s">
+      <c r="A3" s="19" t="s">
         <v>13</v>
       </c>
       <c r="B3" t="s">
@@ -672,7 +671,7 @@
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.55000000000000004">
-      <c r="A4" s="18"/>
+      <c r="A4" s="19"/>
       <c r="B4" s="3">
         <v>700</v>
       </c>
@@ -684,7 +683,7 @@
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.55000000000000004">
-      <c r="A6" s="18" t="s">
+      <c r="A6" s="19" t="s">
         <v>12</v>
       </c>
       <c r="B6" t="s">
@@ -701,7 +700,7 @@
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.55000000000000004">
-      <c r="A7" s="18"/>
+      <c r="A7" s="19"/>
       <c r="B7" s="4">
         <v>8.5500000000000007</v>
       </c>
@@ -721,7 +720,7 @@
       <c r="B8" s="3"/>
     </row>
     <row r="9" spans="1:5" ht="14.4" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A9" s="18" t="s">
+      <c r="A9" s="19" t="s">
         <v>11</v>
       </c>
       <c r="B9" t="s">
@@ -735,7 +734,7 @@
       </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.55000000000000004">
-      <c r="A10" s="18"/>
+      <c r="A10" s="19"/>
       <c r="B10" s="5">
         <v>2.7</v>
       </c>
@@ -748,7 +747,7 @@
       <c r="E10" s="14"/>
     </row>
     <row r="12" spans="1:5" ht="14.4" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A12" s="18" t="s">
+      <c r="A12" s="19" t="s">
         <v>14</v>
       </c>
       <c r="B12" t="s">
@@ -762,7 +761,7 @@
       </c>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.55000000000000004">
-      <c r="A13" s="18"/>
+      <c r="A13" s="19"/>
       <c r="B13" s="3">
         <v>20450</v>
       </c>
@@ -780,7 +779,7 @@
       <c r="E14" s="14"/>
     </row>
     <row r="15" spans="1:5" ht="14.4" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A15" s="18" t="s">
+      <c r="A15" s="19" t="s">
         <v>17</v>
       </c>
       <c r="B15" s="2" t="s">
@@ -797,7 +796,7 @@
       </c>
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.55000000000000004">
-      <c r="A16" s="18"/>
+      <c r="A16" s="19"/>
       <c r="B16" s="2">
         <v>120</v>
       </c>
@@ -813,7 +812,7 @@
       </c>
     </row>
     <row r="18" spans="1:4" ht="14.4" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A18" s="18" t="s">
+      <c r="A18" s="19" t="s">
         <v>50</v>
       </c>
       <c r="B18" t="s">
@@ -824,7 +823,7 @@
       </c>
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.55000000000000004">
-      <c r="A19" s="18"/>
+      <c r="A19" s="19"/>
       <c r="B19" s="7">
         <f>((B16+C16) / C13) + E16</f>
         <v>3.4938875305623474</v>
@@ -835,7 +834,7 @@
       </c>
     </row>
     <row r="21" spans="1:4" ht="14.4" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A21" s="18" t="s">
+      <c r="A21" s="19" t="s">
         <v>22</v>
       </c>
       <c r="B21" s="2" t="s">
@@ -846,17 +845,17 @@
       </c>
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.55000000000000004">
-      <c r="A22" s="18"/>
+      <c r="A22" s="19"/>
       <c r="B22" s="9">
-        <v>20</v>
+        <v>0</v>
       </c>
       <c r="C22" s="9">
         <f>B22/60</f>
-        <v>0.33333333333333331</v>
+        <v>0</v>
       </c>
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.55000000000000004">
-      <c r="A24" s="18" t="s">
+      <c r="A24" s="19" t="s">
         <v>23</v>
       </c>
       <c r="B24" s="2" t="s">
@@ -870,22 +869,22 @@
       </c>
     </row>
     <row r="25" spans="1:4" x14ac:dyDescent="0.55000000000000004">
-      <c r="A25" s="18"/>
+      <c r="A25" s="19"/>
       <c r="B25" s="10">
         <f>B16*C22</f>
-        <v>40</v>
+        <v>0</v>
       </c>
       <c r="C25" s="11">
         <f>C22*C16</f>
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="D25" s="12">
         <f>C22*E16</f>
-        <v>0.33333333333333331</v>
+        <v>0</v>
       </c>
     </row>
     <row r="27" spans="1:4" x14ac:dyDescent="0.55000000000000004">
-      <c r="A27" s="18" t="s">
+      <c r="A27" s="19" t="s">
         <v>55</v>
       </c>
       <c r="B27" t="s">
@@ -896,7 +895,7 @@
       </c>
     </row>
     <row r="28" spans="1:4" x14ac:dyDescent="0.55000000000000004">
-      <c r="A28" s="18"/>
+      <c r="A28" s="19"/>
       <c r="B28">
         <v>10</v>
       </c>
@@ -906,7 +905,7 @@
       </c>
     </row>
     <row r="30" spans="1:4" ht="14.4" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A30" s="18" t="s">
+      <c r="A30" s="19" t="s">
         <v>16</v>
       </c>
       <c r="B30" t="s">
@@ -917,57 +916,57 @@
       </c>
     </row>
     <row r="31" spans="1:4" x14ac:dyDescent="0.55000000000000004">
-      <c r="A31" s="18"/>
+      <c r="A31" s="19"/>
       <c r="B31" s="13">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="C31" s="11">
         <f>B31*C13</f>
-        <v>902.20588235294122</v>
+        <v>601.47058823529414</v>
       </c>
     </row>
     <row r="33" spans="1:3" x14ac:dyDescent="0.55000000000000004">
-      <c r="A33" s="18" t="s">
+      <c r="A33" s="19" t="s">
         <v>37</v>
       </c>
       <c r="B33" t="s">
+        <v>36</v>
+      </c>
+      <c r="C33" t="s">
         <v>38</v>
       </c>
-      <c r="C33" t="s">
-        <v>36</v>
-      </c>
     </row>
     <row r="34" spans="1:3" x14ac:dyDescent="0.55000000000000004">
-      <c r="A34" s="18"/>
-      <c r="B34" s="11">
-        <f>C34*C13</f>
-        <v>501.12299019607849</v>
-      </c>
-      <c r="C34" s="16">
+      <c r="A34" s="19"/>
+      <c r="B34" s="16">
         <f>D13 +B10 + C10 +D10 +(B25 / C13) + (C25 / C13) +D25</f>
-        <v>8.3316291768541166</v>
+        <v>7.1669999999999998</v>
+      </c>
+      <c r="C34" s="11">
+        <f>B34*C13</f>
+        <v>431.07397058823528</v>
       </c>
     </row>
     <row r="36" spans="1:3" x14ac:dyDescent="0.55000000000000004">
-      <c r="A36" s="18" t="s">
+      <c r="A36" s="19" t="s">
         <v>15</v>
       </c>
       <c r="B36" t="s">
+        <v>30</v>
+      </c>
+      <c r="C36" t="s">
         <v>29</v>
       </c>
-      <c r="C36" t="s">
-        <v>30</v>
-      </c>
     </row>
     <row r="37" spans="1:3" x14ac:dyDescent="0.55000000000000004">
-      <c r="A37" s="18"/>
+      <c r="A37" s="19"/>
       <c r="B37" s="11">
-        <f>(C13*B31) - B34</f>
-        <v>401.08289215686273</v>
+        <f>B31-B34</f>
+        <v>2.8330000000000002</v>
       </c>
       <c r="C37" s="11">
-        <f>B31-C34</f>
-        <v>6.6683708231458834</v>
+        <f>(C13*B31) - C34</f>
+        <v>170.39661764705886</v>
       </c>
     </row>
     <row r="38" spans="1:3" x14ac:dyDescent="0.55000000000000004">
@@ -977,7 +976,7 @@
       <c r="C38" s="20"/>
     </row>
     <row r="39" spans="1:3" x14ac:dyDescent="0.55000000000000004">
-      <c r="A39" s="18" t="s">
+      <c r="A39" s="19" t="s">
         <v>32</v>
       </c>
       <c r="B39" t="s">
@@ -985,38 +984,38 @@
       </c>
     </row>
     <row r="40" spans="1:3" x14ac:dyDescent="0.55000000000000004">
-      <c r="A40" s="18"/>
+      <c r="A40" s="19"/>
       <c r="B40" s="14">
         <v>0.5</v>
       </c>
     </row>
     <row r="42" spans="1:3" x14ac:dyDescent="0.55000000000000004">
-      <c r="A42" s="18" t="s">
+      <c r="A42" s="19" t="s">
         <v>33</v>
       </c>
       <c r="B42" t="s">
+        <v>30</v>
+      </c>
+      <c r="C42" t="s">
         <v>29</v>
       </c>
-      <c r="C42" t="s">
-        <v>30</v>
-      </c>
     </row>
     <row r="43" spans="1:3" x14ac:dyDescent="0.55000000000000004">
-      <c r="A43" s="18"/>
+      <c r="A43" s="19"/>
       <c r="B43" s="11">
         <f>B37*B40</f>
-        <v>200.54144607843136</v>
+        <v>1.4165000000000001</v>
       </c>
       <c r="C43" s="11">
         <f>C37*B40</f>
-        <v>3.3341854115729417</v>
+        <v>85.19830882352943</v>
       </c>
     </row>
     <row r="47" spans="1:3" x14ac:dyDescent="0.55000000000000004">
-      <c r="B47" s="19" t="s">
+      <c r="B47" s="18" t="s">
         <v>40</v>
       </c>
-      <c r="C47" s="19"/>
+      <c r="C47" s="18"/>
     </row>
     <row r="48" spans="1:3" x14ac:dyDescent="0.55000000000000004">
       <c r="B48" s="1" t="s">
@@ -1031,8 +1030,8 @@
         <v>43</v>
       </c>
       <c r="C49" s="14">
-        <f>D13/$C$34</f>
-        <v>0.34891135194493073</v>
+        <f>D13/$B$34</f>
+        <v>0.40560904143993304</v>
       </c>
     </row>
     <row r="50" spans="2:3" x14ac:dyDescent="0.55000000000000004">
@@ -1040,8 +1039,8 @@
         <v>45</v>
       </c>
       <c r="C50" s="14">
-        <f>B10/$C$34</f>
-        <v>0.32406627115628239</v>
+        <f>B10/$B$34</f>
+        <v>0.37672666387609882</v>
       </c>
     </row>
     <row r="51" spans="2:3" x14ac:dyDescent="0.55000000000000004">
@@ -1049,8 +1048,8 @@
         <v>44</v>
       </c>
       <c r="C51" s="14">
-        <f>C10/$C$34</f>
-        <v>7.2014726923618306E-3</v>
+        <f>C10/$B$34</f>
+        <v>8.3717036416910834E-3</v>
       </c>
     </row>
     <row r="52" spans="2:3" x14ac:dyDescent="0.55000000000000004">
@@ -1058,8 +1057,8 @@
         <v>57</v>
       </c>
       <c r="C52" s="14">
-        <f>D10/$C$34</f>
-        <v>0.18003681730904578</v>
+        <f>D10/$B$34</f>
+        <v>0.2092925910422771</v>
       </c>
     </row>
     <row r="53" spans="2:3" x14ac:dyDescent="0.55000000000000004">
@@ -1067,8 +1066,8 @@
         <v>58</v>
       </c>
       <c r="C53" s="14">
-        <f>(B25/$C$13)/$C$34</f>
-        <v>7.9820724218517436E-2</v>
+        <f>(B25/$C$13)/$B$34</f>
+        <v>0</v>
       </c>
     </row>
     <row r="54" spans="2:3" x14ac:dyDescent="0.55000000000000004">
@@ -1076,8 +1075,8 @@
         <v>47</v>
       </c>
       <c r="C54" s="15">
-        <f>D25/$C$34</f>
-        <v>4.0008181624232392E-2</v>
+        <f>D25/$B$34</f>
+        <v>0</v>
       </c>
     </row>
     <row r="55" spans="2:3" x14ac:dyDescent="0.55000000000000004">
@@ -1085,8 +1084,8 @@
         <v>46</v>
       </c>
       <c r="C55" s="14">
-        <f>(C25/$C$13)/$C$34</f>
-        <v>1.9955181054629359E-2</v>
+        <f>(C25/$C$13)/$B$34</f>
+        <v>0</v>
       </c>
     </row>
     <row r="56" spans="2:3" x14ac:dyDescent="0.55000000000000004">
@@ -1095,11 +1094,16 @@
       </c>
       <c r="C56" s="14">
         <f>SUM(C49:C55)</f>
-        <v>0.99999999999999989</v>
+        <v>1</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="16">
+    <mergeCell ref="A3:A4"/>
+    <mergeCell ref="A6:A7"/>
+    <mergeCell ref="A9:A10"/>
+    <mergeCell ref="A12:A13"/>
+    <mergeCell ref="A21:A22"/>
     <mergeCell ref="B47:C47"/>
     <mergeCell ref="A18:A19"/>
     <mergeCell ref="A36:A37"/>
@@ -1111,11 +1115,6 @@
     <mergeCell ref="A33:A34"/>
     <mergeCell ref="A27:A28"/>
     <mergeCell ref="A30:A31"/>
-    <mergeCell ref="A3:A4"/>
-    <mergeCell ref="A6:A7"/>
-    <mergeCell ref="A9:A10"/>
-    <mergeCell ref="A12:A13"/>
-    <mergeCell ref="A21:A22"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>